<commit_message>
Add India to production hours billable summary
Adds India across Jul 2025-Jun 2026 (12 LOBs). Sum duplicate LOB rows
within a month to capture catch-up billing (e.g. India WIMS December
additional billing booked in January). Use India October v2 file.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGJRZ14kGC15zQ7YESHNbn
</commit_message>
<xml_diff>
--- a/Production_Hours_Billable_Summary.xlsx
+++ b/Production_Hours_Billable_Summary.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Jamaica" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Egypt" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Canada" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="India" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,11 +478,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -507,7 +508,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: "Production hrs Billing Summary" sheet → "Hrs. Billable" column, LOB Total rows</t>
+          <t>Source: "Production hrs Billing Summary" sheet -&gt; "Hrs. Billable" column, LOB Total rows</t>
         </is>
       </c>
     </row>
@@ -1040,39 +1041,41 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ESL NA LPAX Voice Service - Production</t>
+          <t>ESL NA Digital Sales - Production</t>
         </is>
       </c>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
+      <c r="E15" s="5" t="n">
+        <v>1540.21</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>821.1</v>
+      </c>
       <c r="G15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>3596.36</v>
-      </c>
-      <c r="I15" s="5" t="n">
-        <v>3708.94</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="n"/>
       <c r="J15" s="5" t="n">
-        <v>3097.88</v>
+        <v>1893.36</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>4016.79</v>
+        <v>2478.25</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>4966.04</v>
+        <v>1961.14</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>4310.21</v>
+        <v>2081.7</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>3198.53</v>
+        <v>1747.12</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>26894.75</v>
+        <v>12522.88</v>
       </c>
     </row>
     <row r="16">
@@ -1083,35 +1086,43 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Voice Service - Production</t>
+          <t>CA FR Voice - Production</t>
         </is>
       </c>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
+      <c r="E16" s="5" t="n">
+        <v>2048.13</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>2478.7</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>1669.95</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>3247.74</v>
+      </c>
       <c r="I16" s="5" t="n">
-        <v>997.02</v>
+        <v>1937.85</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>18542.23</v>
+        <v>2864.36</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>21860.94</v>
+        <v>3471.15</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>22695.23</v>
+        <v>3221.71</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>25759.65</v>
+        <v>2471.84</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>26567.43</v>
+        <v>1811.12</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>116422.51</v>
+        <v>25222.55</v>
       </c>
     </row>
     <row r="17">
@@ -1122,43 +1133,43 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CA FR Voice - Production</t>
+          <t>ESL UK Digital Sales - Production</t>
         </is>
       </c>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="5" t="n">
-        <v>2048.13</v>
+        <v>1789.5</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>2478.7</v>
+        <v>0</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>1669.95</v>
+        <v>0</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>3247.74</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>1937.85</v>
+        <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>2864.36</v>
+        <v>0</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>3471.15</v>
+        <v>0</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>3221.71</v>
+        <v>0</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>2471.84</v>
+        <v>0</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>1811.12</v>
+        <v>0</v>
       </c>
       <c r="O17" s="7" t="n">
-        <v>25222.55</v>
+        <v>1789.5</v>
       </c>
     </row>
     <row r="18">
@@ -1169,43 +1180,43 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Digital Sales - Production</t>
+          <t>ESL NA Voice Sales - Production</t>
         </is>
       </c>
       <c r="C18" s="6" t="n"/>
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="5" t="n">
-        <v>1789.5</v>
+        <v>2528.78</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0</v>
+        <v>9166.530000000001</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>0</v>
+        <v>10549.24</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0</v>
+        <v>11047.94</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>0</v>
+        <v>12212.02</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0</v>
+        <v>9152.17</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>0</v>
+        <v>13455.47</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>0</v>
+        <v>14566.36</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>0</v>
+        <v>13823.69</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0</v>
+        <v>9621.950000000001</v>
       </c>
       <c r="O18" s="7" t="n">
-        <v>1789.5</v>
+        <v>106124.15</v>
       </c>
     </row>
     <row r="19">
@@ -1216,43 +1227,43 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Voice Sales - Production</t>
+          <t>ESL UK Voice Service - Production</t>
         </is>
       </c>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="5" t="n">
-        <v>2528.78</v>
+        <v>2971.44</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>9166.530000000001</v>
+        <v>2816.31</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>10549.24</v>
+        <v>4180.76</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>11047.94</v>
+        <v>4675.02</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>12212.02</v>
+        <v>5582.91</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>9152.17</v>
+        <v>4007.21</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>13455.47</v>
+        <v>6752.89</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>14566.36</v>
+        <v>5759.17</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>13823.69</v>
+        <v>6463.72</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>9621.950000000001</v>
+        <v>4931.92</v>
       </c>
       <c r="O19" s="7" t="n">
-        <v>106124.15</v>
+        <v>48141.35</v>
       </c>
     </row>
     <row r="20">
@@ -1263,43 +1274,43 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Service - Production</t>
+          <t>ESL UK Voice Sales - Production</t>
         </is>
       </c>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="5" t="n">
-        <v>2971.44</v>
+        <v>2171.57</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>2816.31</v>
+        <v>3608.53</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>4180.76</v>
+        <v>2855.1</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>4675.02</v>
+        <v>2309.62</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>5582.91</v>
+        <v>2985.3</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>4007.21</v>
+        <v>1802.92</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>6752.89</v>
+        <v>2027.5</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>5759.17</v>
+        <v>2092.43</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>6463.72</v>
+        <v>1716.88</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>4931.92</v>
+        <v>1276.85</v>
       </c>
       <c r="O20" s="7" t="n">
-        <v>48141.35</v>
+        <v>22846.7</v>
       </c>
     </row>
     <row r="21">
@@ -1310,43 +1321,43 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Sales - Production</t>
+          <t>ESL SP Voice Service - Production</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="5" t="n">
-        <v>2171.57</v>
+        <v>876.1799999999999</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>3608.53</v>
+        <v>2608.21</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>2855.1</v>
+        <v>2282.77</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>2309.62</v>
+        <v>3582.5</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>2985.3</v>
+        <v>2520.79</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>1802.92</v>
+        <v>3094.4</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2027.5</v>
+        <v>3435.69</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>2092.43</v>
+        <v>3161.93</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>1716.88</v>
+        <v>2525.53</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>1276.85</v>
+        <v>1651.05</v>
       </c>
       <c r="O21" s="7" t="n">
-        <v>22846.7</v>
+        <v>25739.05</v>
       </c>
     </row>
     <row r="22">
@@ -1357,43 +1368,39 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>ESL SP Voice Service - Production</t>
+          <t>ESL NA LPAX Voice Service - Production</t>
         </is>
       </c>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
-      <c r="E22" s="5" t="n">
-        <v>876.1799999999999</v>
-      </c>
-      <c r="F22" s="5" t="n">
-        <v>2608.21</v>
-      </c>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
       <c r="G22" s="5" t="n">
-        <v>2282.77</v>
+        <v>0</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>3582.5</v>
+        <v>6183.13</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>2520.79</v>
+        <v>3708.94</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>3094.4</v>
+        <v>3097.88</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>3435.69</v>
+        <v>4016.79</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>3161.93</v>
+        <v>4966.04</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>2525.53</v>
+        <v>4310.21</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>1651.05</v>
+        <v>3198.53</v>
       </c>
       <c r="O22" s="7" t="n">
-        <v>25739.05</v>
+        <v>29481.52</v>
       </c>
     </row>
     <row r="23">
@@ -1404,39 +1411,35 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Service DHD - Production</t>
+          <t>ESL NA Voice Service - Production</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
-      <c r="G23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>501.48</v>
-      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
       <c r="I23" s="5" t="n">
-        <v>2173.77</v>
+        <v>997.02</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>3109.29</v>
+        <v>18542.23</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>2488.02</v>
+        <v>21860.94</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>2239.05</v>
+        <v>22695.23</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>2544.9</v>
+        <v>25759.65</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>2334.82</v>
+        <v>26567.43</v>
       </c>
       <c r="O23" s="7" t="n">
-        <v>15391.33</v>
+        <v>116422.51</v>
       </c>
     </row>
     <row r="24">
@@ -1447,41 +1450,39 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Digital Sales - Production</t>
+          <t>ESL UK Voice Service DHD - Production</t>
         </is>
       </c>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
-      <c r="E24" s="5" t="n">
-        <v>1540.21</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>821.1</v>
-      </c>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
       <c r="G24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="6" t="n"/>
+        <v>1936.91</v>
+      </c>
+      <c r="I24" s="5" t="n">
+        <v>2173.77</v>
+      </c>
       <c r="J24" s="5" t="n">
-        <v>1893.36</v>
+        <v>3109.29</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>2478.25</v>
+        <v>2488.02</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>1961.14</v>
+        <v>2239.05</v>
       </c>
       <c r="M24" s="5" t="n">
-        <v>2081.7</v>
+        <v>2544.9</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>1747.12</v>
+        <v>2334.82</v>
       </c>
       <c r="O24" s="7" t="n">
-        <v>12522.88</v>
+        <v>16826.76</v>
       </c>
     </row>
     <row r="25">
@@ -1653,7 +1654,7 @@
         <v>48276.24</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>54496.13</v>
+        <v>58518.33</v>
       </c>
       <c r="I29" s="9" t="n">
         <v>61268.47</v>
@@ -1674,7 +1675,7 @@
         <v>71491.75</v>
       </c>
       <c r="O29" s="9" t="n">
-        <v>666768.74</v>
+        <v>670790.9399999999</v>
       </c>
     </row>
     <row r="30">
@@ -1767,38 +1768,610 @@
         <v>10519.58</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>CSO - Production</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>4197.42</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>3664.6</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>2738.91</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>2457.4</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>2142.5</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>2515.43</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>2417.13</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>2293.84</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>1821.57</v>
+      </c>
+      <c r="L32" s="6" t="n"/>
+      <c r="M32" s="5" t="n">
+        <v>1343.95</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>1346.02</v>
+      </c>
+      <c r="O32" s="7" t="n">
+        <v>26938.76</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>LPS - Production</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>4259.47</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>3716.68</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>3512.8</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>3901.6</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>3192.49</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>3649.14</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>4025.44</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>3353</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>4049.53</v>
+      </c>
+      <c r="L33" s="6" t="n"/>
+      <c r="M33" s="5" t="n">
+        <v>3701.64</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>3228.58</v>
+      </c>
+      <c r="O33" s="7" t="n">
+        <v>40590.38</v>
+      </c>
+    </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>NA Frontline - Production</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>16273.82</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>24548.62</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>34857.61</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>36645.12</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>48700.41</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>48180.59</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>42471.29</v>
+      </c>
+      <c r="J34" s="5" t="n">
+        <v>38283.74</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>49252.73</v>
+      </c>
+      <c r="L34" s="6" t="n"/>
+      <c r="M34" s="5" t="n">
+        <v>46958.48</v>
+      </c>
+      <c r="N34" s="5" t="n">
+        <v>37271.87</v>
+      </c>
+      <c r="O34" s="7" t="n">
+        <v>423444.27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>WIMS - Production</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>2267</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>2347.5</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>2194.29</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>2446.57</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>2267.4</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>2267.43</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>2555.71</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>2078.97</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>2435.78</v>
+      </c>
+      <c r="L35" s="6" t="n"/>
+      <c r="M35" s="5" t="n">
+        <v>2267.43</v>
+      </c>
+      <c r="N35" s="5" t="n">
+        <v>1920.22</v>
+      </c>
+      <c r="O35" s="7" t="n">
+        <v>25048.29</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Permitted Adjustments</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>4259.55</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>3232.15</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>3874.29</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>7363.5</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>7212.28</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>10333.09</v>
+      </c>
+      <c r="I36" s="5" t="n">
+        <v>10537.49</v>
+      </c>
+      <c r="J36" s="5" t="n">
+        <v>11541.01</v>
+      </c>
+      <c r="K36" s="5" t="n">
+        <v>15754.05</v>
+      </c>
+      <c r="L36" s="6" t="n"/>
+      <c r="M36" s="5" t="n">
+        <v>15019.9</v>
+      </c>
+      <c r="N36" s="5" t="n">
+        <v>12439.23</v>
+      </c>
+      <c r="O36" s="7" t="n">
+        <v>101566.54</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Digital Sales</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="5" t="n">
+        <v>3182.23</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>5513.37</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>6583.62</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>5919.16</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>5967.17</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>8911.450000000001</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>14637.92</v>
+      </c>
+      <c r="L37" s="6" t="n"/>
+      <c r="M37" s="5" t="n">
+        <v>12148.64</v>
+      </c>
+      <c r="N37" s="5" t="n">
+        <v>8313.15</v>
+      </c>
+      <c r="O37" s="7" t="n">
+        <v>71176.71000000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Customer Payments</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="5" t="n">
+        <v>758.5700000000001</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>805.42</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>531.4</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>531.4299999999999</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <v>611.4</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <v>496.74</v>
+      </c>
+      <c r="K38" s="5" t="n">
+        <v>569.73</v>
+      </c>
+      <c r="L38" s="6" t="n"/>
+      <c r="M38" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="N38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="7" t="n">
+        <v>4336.69</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>WFM Support</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="5" t="n">
+        <v>256</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>312</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>458.3</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="K39" s="5" t="n">
+        <v>394.3</v>
+      </c>
+      <c r="L39" s="6" t="n"/>
+      <c r="M39" s="5" t="n">
+        <v>354.29</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>382.86</v>
+      </c>
+      <c r="O39" s="7" t="n">
+        <v>2777.74</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>NA RPOps &amp; STOps</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <v>6876.42</v>
+      </c>
+      <c r="L40" s="5" t="n">
+        <v>6733.52</v>
+      </c>
+      <c r="M40" s="6" t="n"/>
+      <c r="N40" s="5" t="n">
+        <v>6405.72</v>
+      </c>
+      <c r="O40" s="7" t="n">
+        <v>20015.65</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>RMT - Production</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>1608.72</v>
+      </c>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="n"/>
+      <c r="J41" s="6" t="n"/>
+      <c r="K41" s="6" t="n"/>
+      <c r="L41" s="6" t="n"/>
+      <c r="M41" s="6" t="n"/>
+      <c r="N41" s="6" t="n"/>
+      <c r="O41" s="7" t="n">
+        <v>1608.72</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Finance Team</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="5" t="n">
+        <v>739.9</v>
+      </c>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
+      <c r="J42" s="6" t="n"/>
+      <c r="K42" s="6" t="n"/>
+      <c r="L42" s="6" t="n"/>
+      <c r="M42" s="6" t="n"/>
+      <c r="N42" s="6" t="n"/>
+      <c r="O42" s="7" t="n">
+        <v>739.9</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>NA Analytics</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="6" t="n"/>
+      <c r="J43" s="6" t="n"/>
+      <c r="K43" s="6" t="n"/>
+      <c r="L43" s="6" t="n"/>
+      <c r="M43" s="6" t="n"/>
+      <c r="N43" s="5" t="n">
+        <v>944</v>
+      </c>
+      <c r="O43" s="7" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>India Total</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="n">
+        <v>32865.97</v>
+      </c>
+      <c r="D44" s="9" t="n">
+        <v>38249.45</v>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>51118.69</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>59388.98</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>70930.10000000001</v>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>73708.27</v>
+      </c>
+      <c r="I44" s="9" t="n">
+        <v>69043.92999999999</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>67278.75</v>
+      </c>
+      <c r="K44" s="9" t="n">
+        <v>95792.03</v>
+      </c>
+      <c r="L44" s="9" t="n">
+        <v>6733.52</v>
+      </c>
+      <c r="M44" s="9" t="n">
+        <v>81826.34</v>
+      </c>
+      <c r="N44" s="9" t="n">
+        <v>72251.64</v>
+      </c>
+      <c r="O44" s="9" t="n">
+        <v>719187.66</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>• Values = "Hrs. Billable" total for each LOB (column G in 2025 files / column F in 2026 files; located by header).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>• Jamaica: December 2025 not provided; February 2026 file is B2C-only (other LOBs blank in source).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>• Canada: only September 2025 - February 2026 provided.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>• Blank cell = LOB not present / no data in that month's file.</t>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>- Values = "Hrs. Billable" total per LOB (col G in 2025 files / col F in 2026 files; located by header).</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>- Duplicate LOB rows within a month (e.g. India WIMS "additional billing" catch-up) are summed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>- Jamaica: Dec 2025 not provided; Feb 2026 file is B2C-only (other LOBs blank).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>- Canada: only Sep 2025 - Feb 2026 provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>- India: Apr 2026 file is GPS/RPOps-only - only "NA RPOps &amp; STOps" populated; service LOBs blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>- India Oct 2025: used the v2 (revised) file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>- Blank cell = LOB not present / no data in that month file.</t>
         </is>
       </c>
     </row>
@@ -1816,7 +2389,7 @@
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -1834,7 +2407,7 @@
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Jamaica — Production Hours Billable by LOB and Month</t>
+          <t>Jamaica - Production Hours Billable by LOB and Month</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2784,7 @@
   <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -2230,7 +2803,7 @@
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Egypt — Production Hours Billable by LOB and Month</t>
+          <t>Egypt - Production Hours Billable by LOB and Month</t>
         </is>
       </c>
     </row>
@@ -2401,403 +2974,403 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>ESL NA LPAX Voice Service - Production</t>
+          <t>ESL NA Digital Sales - Production</t>
         </is>
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
+      <c r="D6" s="5" t="n">
+        <v>1540.21</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>821.1</v>
+      </c>
       <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>3596.36</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>3708.94</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H6" s="6" t="n"/>
       <c r="I6" s="5" t="n">
-        <v>3097.88</v>
+        <v>1893.36</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>4016.79</v>
+        <v>2478.25</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>4966.04</v>
+        <v>1961.14</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>4310.21</v>
+        <v>2081.7</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>3198.53</v>
+        <v>1747.12</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>26894.75</v>
+        <v>12522.88</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Voice Service - Production</t>
+          <t>CA FR Voice - Production</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
+      <c r="D7" s="5" t="n">
+        <v>2048.13</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2478.7</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1669.95</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>3247.74</v>
+      </c>
       <c r="H7" s="5" t="n">
-        <v>997.02</v>
+        <v>1937.85</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>18542.23</v>
+        <v>2864.36</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>21860.94</v>
+        <v>3471.15</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>22695.23</v>
+        <v>3221.71</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>25759.65</v>
+        <v>2471.84</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>26567.43</v>
+        <v>1811.12</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>116422.51</v>
+        <v>25222.55</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CA FR Voice - Production</t>
+          <t>ESL UK Digital Sales - Production</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="5" t="n">
-        <v>2048.13</v>
+        <v>1789.5</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>2478.7</v>
+        <v>0</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>1669.95</v>
+        <v>0</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>3247.74</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>1937.85</v>
+        <v>0</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>2864.36</v>
+        <v>0</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>3471.15</v>
+        <v>0</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>3221.71</v>
+        <v>0</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>2471.84</v>
+        <v>0</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>1811.12</v>
+        <v>0</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>25222.55</v>
+        <v>1789.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Digital Sales - Production</t>
+          <t>ESL NA Voice Sales - Production</t>
         </is>
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="5" t="n">
-        <v>1789.5</v>
+        <v>2528.78</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0</v>
+        <v>9166.530000000001</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>10549.24</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0</v>
+        <v>11047.94</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0</v>
+        <v>12212.02</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0</v>
+        <v>9152.17</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0</v>
+        <v>13455.47</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0</v>
+        <v>14566.36</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0</v>
+        <v>13823.69</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>0</v>
+        <v>9621.950000000001</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>1789.5</v>
+        <v>106124.15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Voice Sales - Production</t>
+          <t>ESL UK Voice Service - Production</t>
         </is>
       </c>
       <c r="B10" s="6" t="n"/>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="5" t="n">
-        <v>2528.78</v>
+        <v>2971.44</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>9166.530000000001</v>
+        <v>2816.31</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>10549.24</v>
+        <v>4180.76</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>11047.94</v>
+        <v>4675.02</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>12212.02</v>
+        <v>5582.91</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>9152.17</v>
+        <v>4007.21</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>13455.47</v>
+        <v>6752.89</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>14566.36</v>
+        <v>5759.17</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>13823.69</v>
+        <v>6463.72</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>9621.950000000001</v>
+        <v>4931.92</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>106124.15</v>
+        <v>48141.35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Service - Production</t>
+          <t>ESL UK Voice Sales - Production</t>
         </is>
       </c>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="5" t="n">
-        <v>2971.44</v>
+        <v>2171.57</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>2816.31</v>
+        <v>3608.53</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>4180.76</v>
+        <v>2855.1</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>4675.02</v>
+        <v>2309.62</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>5582.91</v>
+        <v>2985.3</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>4007.21</v>
+        <v>1802.92</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>6752.89</v>
+        <v>2027.5</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>5759.17</v>
+        <v>2092.43</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>6463.72</v>
+        <v>1716.88</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>4931.92</v>
+        <v>1276.85</v>
       </c>
       <c r="N11" s="7" t="n">
-        <v>48141.35</v>
+        <v>22846.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Sales - Production</t>
+          <t>ESL SP Voice Service - Production</t>
         </is>
       </c>
       <c r="B12" s="6" t="n"/>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="5" t="n">
-        <v>2171.57</v>
+        <v>876.1799999999999</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>3608.53</v>
+        <v>2608.21</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>2855.1</v>
+        <v>2282.77</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>2309.62</v>
+        <v>3582.5</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>2985.3</v>
+        <v>2520.79</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>1802.92</v>
+        <v>3094.4</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>2027.5</v>
+        <v>3435.69</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>2092.43</v>
+        <v>3161.93</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>1716.88</v>
+        <v>2525.53</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>1276.85</v>
+        <v>1651.05</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>22846.7</v>
+        <v>25739.05</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>ESL SP Voice Service - Production</t>
+          <t>ESL NA LPAX Voice Service - Production</t>
         </is>
       </c>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
-      <c r="D13" s="5" t="n">
-        <v>876.1799999999999</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>2608.21</v>
-      </c>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
       <c r="F13" s="5" t="n">
-        <v>2282.77</v>
+        <v>0</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>3582.5</v>
+        <v>6183.13</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2520.79</v>
+        <v>3708.94</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>3094.4</v>
+        <v>3097.88</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>3435.69</v>
+        <v>4016.79</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>3161.93</v>
+        <v>4966.04</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>2525.53</v>
+        <v>4310.21</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>1651.05</v>
+        <v>3198.53</v>
       </c>
       <c r="N13" s="7" t="n">
-        <v>25739.05</v>
+        <v>29481.52</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Service DHD - Production</t>
+          <t>ESL NA Voice Service - Production</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
-      <c r="F14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>501.48</v>
-      </c>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
       <c r="H14" s="5" t="n">
-        <v>2173.77</v>
+        <v>997.02</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>3109.29</v>
+        <v>18542.23</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>2488.02</v>
+        <v>21860.94</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>2239.05</v>
+        <v>22695.23</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>2544.9</v>
+        <v>25759.65</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>2334.82</v>
+        <v>26567.43</v>
       </c>
       <c r="N14" s="7" t="n">
-        <v>15391.33</v>
+        <v>116422.51</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Digital Sales - Production</t>
+          <t>ESL UK Voice Service DHD - Production</t>
         </is>
       </c>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="5" t="n">
-        <v>1540.21</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>821.1</v>
-      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
       <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="6" t="n"/>
+        <v>1936.91</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>2173.77</v>
+      </c>
       <c r="I15" s="5" t="n">
-        <v>1893.36</v>
+        <v>3109.29</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>2478.25</v>
+        <v>2488.02</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>1961.14</v>
+        <v>2239.05</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>2081.7</v>
+        <v>2544.9</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>1747.12</v>
+        <v>2334.82</v>
       </c>
       <c r="N15" s="7" t="n">
-        <v>12522.88</v>
+        <v>16826.76</v>
       </c>
     </row>
     <row r="16">
@@ -2944,7 +3517,7 @@
         <v>48276.24</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>54496.13</v>
+        <v>58518.33</v>
       </c>
       <c r="H20" s="9" t="n">
         <v>61268.47</v>
@@ -2965,7 +3538,7 @@
         <v>71491.75</v>
       </c>
       <c r="N20" s="9" t="n">
-        <v>666768.74</v>
+        <v>670790.9399999999</v>
       </c>
     </row>
   </sheetData>
@@ -2982,7 +3555,7 @@
   <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -2995,7 +3568,7 @@
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Canada — Production Hours Billable by LOB and Month</t>
+          <t>Canada - Production Hours Billable by LOB and Month</t>
         </is>
       </c>
     </row>
@@ -3095,6 +3668,601 @@
       </c>
       <c r="H5" s="9" t="n">
         <v>10519.58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>India - Production Hours Billable by LOB and Month</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>LOB</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>July 2025</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>August 2025</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>September 2025</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>October 2025</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>November 2025</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>December 2025</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>January 2026</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>February 2026</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>April 2026</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CSO - Production</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>4197.42</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>3664.6</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>2738.91</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>2457.4</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>2142.5</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>2515.43</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>2417.13</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>2293.84</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>1821.57</v>
+      </c>
+      <c r="K4" s="6" t="n"/>
+      <c r="L4" s="5" t="n">
+        <v>1343.95</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>1346.02</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>26938.76</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>LPS - Production</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>4259.47</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>3716.68</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>3512.8</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3901.6</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>3192.49</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>3649.14</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>4025.44</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>3353</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>4049.53</v>
+      </c>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="5" t="n">
+        <v>3701.64</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>3228.58</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>40590.38</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>NA Frontline - Production</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>16273.82</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>24548.62</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>34857.61</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>36645.12</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>48700.41</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>48180.59</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>42471.29</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>38283.74</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>49252.73</v>
+      </c>
+      <c r="K6" s="6" t="n"/>
+      <c r="L6" s="5" t="n">
+        <v>46958.48</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>37271.87</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>423444.27</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>WIMS - Production</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>2267</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>2347.5</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>2194.29</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>2446.57</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2267.4</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>2267.43</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>2555.71</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>2078.97</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>2435.78</v>
+      </c>
+      <c r="K7" s="6" t="n"/>
+      <c r="L7" s="5" t="n">
+        <v>2267.43</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>1920.22</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>25048.29</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Permitted Adjustments</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>4259.55</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>3232.15</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>3874.29</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>7363.5</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>7212.28</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>10333.09</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>10537.49</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>11541.01</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>15754.05</v>
+      </c>
+      <c r="K8" s="6" t="n"/>
+      <c r="L8" s="5" t="n">
+        <v>15019.9</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>12439.23</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>101566.54</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Digital Sales</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="5" t="n">
+        <v>3182.23</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>5513.37</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>6583.62</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>5919.16</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>5967.17</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>8911.450000000001</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>14637.92</v>
+      </c>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="5" t="n">
+        <v>12148.64</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>8313.15</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>71176.71000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Customer Payments</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="5" t="n">
+        <v>758.5700000000001</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>805.42</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>531.4</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>531.4299999999999</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>611.4</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>496.74</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>569.73</v>
+      </c>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>4336.69</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>WFM Support</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="5" t="n">
+        <v>256</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>300</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>312</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>458.3</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>320</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>394.3</v>
+      </c>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="5" t="n">
+        <v>354.29</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>382.86</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>2777.74</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>NA RPOps &amp; STOps</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>6876.42</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>6733.52</v>
+      </c>
+      <c r="L12" s="6" t="n"/>
+      <c r="M12" s="5" t="n">
+        <v>6405.72</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>20015.65</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>RMT - Production</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1608.72</v>
+      </c>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+      <c r="M13" s="6" t="n"/>
+      <c r="N13" s="7" t="n">
+        <v>1608.72</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Finance Team</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="5" t="n">
+        <v>739.9</v>
+      </c>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="n"/>
+      <c r="L14" s="6" t="n"/>
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="7" t="n">
+        <v>739.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>NA Analytics</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="M15" s="5" t="n">
+        <v>944</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>32865.97</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>38249.45</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>51118.69</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>59388.98</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>70930.10000000001</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>73708.27</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>69043.92999999999</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>67278.75</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>95792.03</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>6733.52</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>81826.34</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>72251.64</v>
+      </c>
+      <c r="N16" s="9" t="n">
+        <v>719187.66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Drop all-zero LOB rows and render blanks as zero
Removes LOBs that are zero across all months (e.g. Egypt GPS, Jamaica
WIMS) and fills empty cells with 0.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JGJRZ14kGC15zQ7YESHNbn
</commit_message>
<xml_diff>
--- a/Production_Hours_Billable_Summary.xlsx
+++ b/Production_Hours_Billable_Summary.xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -103,9 +103,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -478,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:O50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -615,11 +612,15 @@
       <c r="G5" s="5" t="n">
         <v>72479.48</v>
       </c>
-      <c r="H5" s="6" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" s="5" t="n">
         <v>59150.74</v>
       </c>
-      <c r="J5" s="6" t="n"/>
+      <c r="J5" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="K5" s="5" t="n">
         <v>43959.67</v>
       </c>
@@ -632,7 +633,7 @@
       <c r="N5" s="5" t="n">
         <v>33943.17</v>
       </c>
-      <c r="O5" s="7" t="n">
+      <c r="O5" s="6" t="n">
         <v>442918.69</v>
       </c>
     </row>
@@ -662,11 +663,15 @@
       <c r="G6" s="5" t="n">
         <v>8782.98</v>
       </c>
-      <c r="H6" s="6" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" s="5" t="n">
         <v>7390.85</v>
       </c>
-      <c r="J6" s="6" t="n"/>
+      <c r="J6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="K6" s="5" t="n">
         <v>5300.01</v>
       </c>
@@ -679,7 +684,7 @@
       <c r="N6" s="5" t="n">
         <v>145.97</v>
       </c>
-      <c r="O6" s="7" t="n">
+      <c r="O6" s="6" t="n">
         <v>100444.69</v>
       </c>
     </row>
@@ -709,11 +714,15 @@
       <c r="G7" s="5" t="n">
         <v>6563.41</v>
       </c>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" s="5" t="n">
         <v>7964.95</v>
       </c>
-      <c r="J7" s="6" t="n"/>
+      <c r="J7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="K7" s="5" t="n">
         <v>9913.139999999999</v>
       </c>
@@ -726,7 +735,7 @@
       <c r="N7" s="5" t="n">
         <v>7413.2</v>
       </c>
-      <c r="O7" s="7" t="n">
+      <c r="O7" s="6" t="n">
         <v>66573.32000000001</v>
       </c>
     </row>
@@ -756,11 +765,15 @@
       <c r="G8" s="5" t="n">
         <v>5399.3</v>
       </c>
-      <c r="H8" s="6" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="5" t="n">
         <v>4194.25</v>
       </c>
-      <c r="J8" s="6" t="n"/>
+      <c r="J8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="K8" s="5" t="n">
         <v>4833.93</v>
       </c>
@@ -773,7 +786,7 @@
       <c r="N8" s="5" t="n">
         <v>10320.62</v>
       </c>
-      <c r="O8" s="7" t="n">
+      <c r="O8" s="6" t="n">
         <v>58307.27</v>
       </c>
     </row>
@@ -788,18 +801,30 @@
           <t>NA LPAX Voice - Production</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" s="5" t="n">
         <v>2881.93</v>
       </c>
-      <c r="H9" s="6" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" s="5" t="n">
         <v>3761.51</v>
       </c>
-      <c r="J9" s="6" t="n"/>
+      <c r="J9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="K9" s="5" t="n">
         <v>3714.27</v>
       </c>
@@ -812,7 +837,7 @@
       <c r="N9" s="5" t="n">
         <v>4713.46</v>
       </c>
-      <c r="O9" s="7" t="n">
+      <c r="O9" s="6" t="n">
         <v>20763.51</v>
       </c>
     </row>
@@ -827,13 +852,27 @@
           <t>B2C - Production</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J10" s="5" t="n">
         <v>1622.5</v>
       </c>
@@ -846,89 +885,113 @@
       <c r="M10" s="5" t="n">
         <v>1038.75</v>
       </c>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="7" t="n">
+      <c r="N10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="6" t="n">
         <v>3164.33</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Jamaica</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>WIMS - Production</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="n"/>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="n"/>
-      <c r="O11" s="7" t="n">
-        <v>0</v>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Jamaica Total</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>60570.3</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>60849.45</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>59022.47</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>68545.72</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>96107.10000000001</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>82462.3</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>1622.5</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>68063.92</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>72325.08</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>66066.56</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>56536.41</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>692171.8100000001</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Jamaica</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Jamaica Total</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>60570.3</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>60849.45</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>59022.47</v>
-      </c>
-      <c r="F12" s="9" t="n">
-        <v>68545.72</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>96107.10000000001</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="9" t="n">
-        <v>82462.3</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>1622.5</v>
-      </c>
-      <c r="K12" s="9" t="n">
-        <v>68063.92</v>
-      </c>
-      <c r="L12" s="9" t="n">
-        <v>72325.08</v>
-      </c>
-      <c r="M12" s="9" t="n">
-        <v>66066.56</v>
-      </c>
-      <c r="N12" s="9" t="n">
-        <v>56536.41</v>
-      </c>
-      <c r="O12" s="9" t="n">
-        <v>692171.8100000001</v>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ESL NA Digital - Production</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>4644.3</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>3915</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>8447.639999999999</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>15980.08</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>17743.04</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>17489</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>22517.23</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>19435.16</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>20403.89</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>18363.81</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>16746.12</v>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>10879.47</v>
+      </c>
+      <c r="O12" s="6" t="n">
+        <v>176564.73</v>
       </c>
     </row>
     <row r="13">
@@ -939,47 +1002,47 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Digital - Production</t>
+          <t>ESL UK Digital - Production</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>4644.3</v>
+        <v>2309.47</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>3915</v>
+        <v>2134</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>8447.639999999999</v>
+        <v>4072.45</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>15980.08</v>
+        <v>6027.18</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>17743.04</v>
+        <v>8995.379999999999</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>17489</v>
+        <v>8046.47</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>22517.23</v>
+        <v>6632.64</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>19435.16</v>
+        <v>6080.16</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>20403.89</v>
+        <v>8569.33</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>18363.81</v>
+        <v>5899.84</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>16746.12</v>
+        <v>5636.43</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>10879.47</v>
-      </c>
-      <c r="O13" s="7" t="n">
-        <v>176564.73</v>
+        <v>4276.37</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>68679.72</v>
       </c>
     </row>
     <row r="14">
@@ -990,47 +1053,47 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Digital - Production</t>
+          <t>ESL NA Digital Sales - Production</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>2309.47</v>
+        <v>0</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2134</v>
+        <v>0</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>4072.45</v>
+        <v>1540.21</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>6027.18</v>
+        <v>821.1</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>8995.379999999999</v>
+        <v>0</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>8046.47</v>
+        <v>0</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>6632.64</v>
+        <v>0</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>6080.16</v>
+        <v>1893.36</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>8569.33</v>
+        <v>2478.25</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>5899.84</v>
+        <v>1961.14</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>5636.43</v>
+        <v>2081.7</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>4276.37</v>
-      </c>
-      <c r="O14" s="7" t="n">
-        <v>68679.72</v>
+        <v>1747.12</v>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>12522.88</v>
       </c>
     </row>
     <row r="15">
@@ -1041,41 +1104,47 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Digital Sales - Production</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
+          <t>CA FR Voice - Production</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E15" s="5" t="n">
-        <v>1540.21</v>
+        <v>2048.13</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>821.1</v>
+        <v>2478.7</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0</v>
+        <v>1669.95</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="6" t="n"/>
+        <v>3247.74</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>1937.85</v>
+      </c>
       <c r="J15" s="5" t="n">
-        <v>1893.36</v>
+        <v>2864.36</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>2478.25</v>
+        <v>3471.15</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>1961.14</v>
+        <v>3221.71</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>2081.7</v>
+        <v>2471.84</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1747.12</v>
-      </c>
-      <c r="O15" s="7" t="n">
-        <v>12522.88</v>
+        <v>1811.12</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>25222.55</v>
       </c>
     </row>
     <row r="16">
@@ -1086,43 +1155,47 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CA FR Voice - Production</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
+          <t>ESL UK Digital Sales - Production</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E16" s="5" t="n">
-        <v>2048.13</v>
+        <v>1789.5</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>2478.7</v>
+        <v>0</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1669.95</v>
+        <v>0</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>3247.74</v>
+        <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>1937.85</v>
+        <v>0</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>2864.36</v>
+        <v>0</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>3471.15</v>
+        <v>0</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>3221.71</v>
+        <v>0</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>2471.84</v>
+        <v>0</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>1811.12</v>
-      </c>
-      <c r="O16" s="7" t="n">
-        <v>25222.55</v>
+        <v>0</v>
+      </c>
+      <c r="O16" s="6" t="n">
+        <v>1789.5</v>
       </c>
     </row>
     <row r="17">
@@ -1133,43 +1206,47 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Digital Sales - Production</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
+          <t>ESL NA Voice Sales - Production</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E17" s="5" t="n">
-        <v>1789.5</v>
+        <v>2528.78</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0</v>
+        <v>9166.530000000001</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0</v>
+        <v>10549.24</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>0</v>
+        <v>11047.94</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0</v>
+        <v>12212.02</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0</v>
+        <v>9152.17</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>0</v>
+        <v>13455.47</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>0</v>
+        <v>14566.36</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>0</v>
+        <v>13823.69</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="7" t="n">
-        <v>1789.5</v>
+        <v>9621.950000000001</v>
+      </c>
+      <c r="O17" s="6" t="n">
+        <v>106124.15</v>
       </c>
     </row>
     <row r="18">
@@ -1180,43 +1257,47 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Voice Sales - Production</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
+          <t>ESL UK Voice Service - Production</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E18" s="5" t="n">
-        <v>2528.78</v>
+        <v>2971.44</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>9166.530000000001</v>
+        <v>2816.31</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>10549.24</v>
+        <v>4180.76</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>11047.94</v>
+        <v>4675.02</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>12212.02</v>
+        <v>5582.91</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>9152.17</v>
+        <v>4007.21</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>13455.47</v>
+        <v>6752.89</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>14566.36</v>
+        <v>5759.17</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>13823.69</v>
+        <v>6463.72</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>9621.950000000001</v>
-      </c>
-      <c r="O18" s="7" t="n">
-        <v>106124.15</v>
+        <v>4931.92</v>
+      </c>
+      <c r="O18" s="6" t="n">
+        <v>48141.35</v>
       </c>
     </row>
     <row r="19">
@@ -1227,43 +1308,47 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Service - Production</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
+          <t>ESL UK Voice Sales - Production</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E19" s="5" t="n">
-        <v>2971.44</v>
+        <v>2171.57</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>2816.31</v>
+        <v>3608.53</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>4180.76</v>
+        <v>2855.1</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>4675.02</v>
+        <v>2309.62</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>5582.91</v>
+        <v>2985.3</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>4007.21</v>
+        <v>1802.92</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>6752.89</v>
+        <v>2027.5</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>5759.17</v>
+        <v>2092.43</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>6463.72</v>
+        <v>1716.88</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>4931.92</v>
-      </c>
-      <c r="O19" s="7" t="n">
-        <v>48141.35</v>
+        <v>1276.85</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>22846.7</v>
       </c>
     </row>
     <row r="20">
@@ -1274,43 +1359,47 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Sales - Production</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
+          <t>ESL SP Voice Service - Production</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E20" s="5" t="n">
-        <v>2171.57</v>
+        <v>876.1799999999999</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>3608.53</v>
+        <v>2608.21</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>2855.1</v>
+        <v>2282.77</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>2309.62</v>
+        <v>3582.5</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>2985.3</v>
+        <v>2520.79</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>1802.92</v>
+        <v>3094.4</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>2027.5</v>
+        <v>3435.69</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>2092.43</v>
+        <v>3161.93</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>1716.88</v>
+        <v>2525.53</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>1276.85</v>
-      </c>
-      <c r="O20" s="7" t="n">
-        <v>22846.7</v>
+        <v>1651.05</v>
+      </c>
+      <c r="O20" s="6" t="n">
+        <v>25739.05</v>
       </c>
     </row>
     <row r="21">
@@ -1321,43 +1410,47 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>ESL SP Voice Service - Production</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
+          <t>ESL NA LPAX Voice Service - Production</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" s="5" t="n">
-        <v>876.1799999999999</v>
+        <v>0</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>2608.21</v>
+        <v>0</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>2282.77</v>
+        <v>0</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>3582.5</v>
+        <v>6183.13</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>2520.79</v>
+        <v>3708.94</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>3094.4</v>
+        <v>3097.88</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>3435.69</v>
+        <v>4016.79</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>3161.93</v>
+        <v>4966.04</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>2525.53</v>
+        <v>4310.21</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>1651.05</v>
-      </c>
-      <c r="O21" s="7" t="n">
-        <v>25739.05</v>
+        <v>3198.53</v>
+      </c>
+      <c r="O21" s="6" t="n">
+        <v>29481.52</v>
       </c>
     </row>
     <row r="22">
@@ -1368,39 +1461,47 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>ESL NA LPAX Voice Service - Production</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
+          <t>ESL NA Voice Service - Production</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>6183.13</v>
+        <v>0</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>3708.94</v>
+        <v>997.02</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>3097.88</v>
+        <v>18542.23</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>4016.79</v>
+        <v>21860.94</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>4966.04</v>
+        <v>22695.23</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>4310.21</v>
+        <v>25759.65</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>3198.53</v>
-      </c>
-      <c r="O22" s="7" t="n">
-        <v>29481.52</v>
+        <v>26567.43</v>
+      </c>
+      <c r="O22" s="6" t="n">
+        <v>116422.51</v>
       </c>
     </row>
     <row r="23">
@@ -1411,35 +1512,47 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>ESL NA Voice Service - Production</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
+          <t>ESL UK Voice Service DHD - Production</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>1936.91</v>
+      </c>
       <c r="I23" s="5" t="n">
-        <v>997.02</v>
+        <v>2173.77</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>18542.23</v>
+        <v>3109.29</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>21860.94</v>
+        <v>2488.02</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>22695.23</v>
+        <v>2239.05</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>25759.65</v>
+        <v>2544.9</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>26567.43</v>
-      </c>
-      <c r="O23" s="7" t="n">
-        <v>116422.51</v>
+        <v>2334.82</v>
+      </c>
+      <c r="O23" s="6" t="n">
+        <v>16826.76</v>
       </c>
     </row>
     <row r="24">
@@ -1450,39 +1563,47 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>ESL UK Voice Service DHD - Production</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
+          <t>French Sales - Production</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="G24" s="5" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>1936.91</v>
+        <v>0</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>2173.77</v>
+        <v>0</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>3109.29</v>
+        <v>839.76</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>2488.02</v>
+        <v>2002.48</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>2239.05</v>
+        <v>1845.12</v>
       </c>
       <c r="M24" s="5" t="n">
-        <v>2544.9</v>
+        <v>1599.37</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>2334.82</v>
-      </c>
-      <c r="O24" s="7" t="n">
-        <v>16826.76</v>
+        <v>1506.23</v>
+      </c>
+      <c r="O24" s="6" t="n">
+        <v>7792.96</v>
       </c>
     </row>
     <row r="25">
@@ -1493,33 +1614,47 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>French Sales - Production</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
+          <t>Spanish Sales - Production</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J25" s="5" t="n">
-        <v>839.76</v>
+        <v>828.1</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>2002.48</v>
+        <v>1985.11</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>1845.12</v>
+        <v>1860.71</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>1599.37</v>
+        <v>1789.7</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>1506.23</v>
-      </c>
-      <c r="O25" s="7" t="n">
-        <v>7792.96</v>
+        <v>1688.9</v>
+      </c>
+      <c r="O25" s="6" t="n">
+        <v>8152.52</v>
       </c>
     </row>
     <row r="26">
@@ -1530,242 +1665,302 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Spanish Sales - Production</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
+          <t>ESL Digital Sales - Production</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>2357.05</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>2127</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J26" s="5" t="n">
-        <v>828.1</v>
+        <v>0</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>1985.11</v>
+        <v>0</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>1860.71</v>
+        <v>0</v>
       </c>
       <c r="M26" s="5" t="n">
-        <v>1789.7</v>
+        <v>0</v>
       </c>
       <c r="N26" s="5" t="n">
-        <v>1688.9</v>
-      </c>
-      <c r="O26" s="7" t="n">
-        <v>8152.52</v>
+        <v>0</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>4484.05</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Egypt</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>GPS - Production</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="7" t="n">
-        <v>0</v>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Egypt Total</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>9310.82</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>8176</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>26445.9</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>43506.64</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>48276.24</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>58518.33</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>61268.47</v>
+      </c>
+      <c r="J27" s="8" t="n">
+        <v>74747</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>92947.50999999999</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>88632.53999999999</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>87469.74000000001</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <v>71491.75</v>
+      </c>
+      <c r="O27" s="8" t="n">
+        <v>670790.9399999999</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>ESL Digital Sales - Production</t>
+          <t>CA Voice - Production</t>
         </is>
       </c>
       <c r="C28" s="5" t="n">
-        <v>2357.05</v>
+        <v>0</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>2127</v>
-      </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-      <c r="M28" s="6" t="n"/>
-      <c r="N28" s="6" t="n"/>
-      <c r="O28" s="7" t="n">
-        <v>4484.05</v>
+        <v>0</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>2073.63</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>2230.7</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>1712</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>2113.83</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>1992.48</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>396.94</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>10519.58</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Egypt Total</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="n">
-        <v>9310.82</v>
-      </c>
-      <c r="D29" s="9" t="n">
-        <v>8176</v>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>26445.9</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <v>43506.64</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>48276.24</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <v>58518.33</v>
-      </c>
-      <c r="I29" s="9" t="n">
-        <v>61268.47</v>
-      </c>
-      <c r="J29" s="9" t="n">
-        <v>74747</v>
-      </c>
-      <c r="K29" s="9" t="n">
-        <v>92947.50999999999</v>
-      </c>
-      <c r="L29" s="9" t="n">
-        <v>88632.53999999999</v>
-      </c>
-      <c r="M29" s="9" t="n">
-        <v>87469.74000000001</v>
-      </c>
-      <c r="N29" s="9" t="n">
-        <v>71491.75</v>
-      </c>
-      <c r="O29" s="9" t="n">
-        <v>670790.9399999999</v>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Canada Total</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>2073.63</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>2230.7</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>1712</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>2113.83</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>1992.48</v>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>396.94</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="8" t="n">
+        <v>10519.58</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>CA Voice - Production</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
+          <t>CSO - Production</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>4197.42</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>3664.6</v>
+      </c>
       <c r="E30" s="5" t="n">
-        <v>2073.63</v>
+        <v>2738.91</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>2230.7</v>
+        <v>2457.4</v>
       </c>
       <c r="G30" s="5" t="n">
-        <v>1712</v>
+        <v>2142.5</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>2113.83</v>
+        <v>2515.43</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>1992.48</v>
+        <v>2417.13</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>396.94</v>
-      </c>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="7" t="n">
-        <v>10519.58</v>
+        <v>2293.84</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>1821.57</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="5" t="n">
+        <v>1343.95</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>1346.02</v>
+      </c>
+      <c r="O30" s="6" t="n">
+        <v>26938.76</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Canada Total</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>2073.63</v>
-      </c>
-      <c r="F31" s="9" t="n">
-        <v>2230.7</v>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>1712</v>
-      </c>
-      <c r="H31" s="9" t="n">
-        <v>2113.83</v>
-      </c>
-      <c r="I31" s="9" t="n">
-        <v>1992.48</v>
-      </c>
-      <c r="J31" s="9" t="n">
-        <v>396.94</v>
-      </c>
-      <c r="K31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" s="9" t="n">
-        <v>10519.58</v>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>LPS - Production</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>4259.47</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>3716.68</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>3512.8</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>3901.6</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>3192.49</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>3649.14</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>4025.44</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>3353</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>4049.53</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>3701.64</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>3228.58</v>
+      </c>
+      <c r="O31" s="6" t="n">
+        <v>40590.38</v>
       </c>
     </row>
     <row r="32">
@@ -1776,45 +1971,47 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>CSO - Production</t>
+          <t>NA Frontline - Production</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>4197.42</v>
+        <v>16273.82</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>3664.6</v>
+        <v>24548.62</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>2738.91</v>
+        <v>34857.61</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>2457.4</v>
+        <v>36645.12</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>2142.5</v>
+        <v>48700.41</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>2515.43</v>
+        <v>48180.59</v>
       </c>
       <c r="I32" s="5" t="n">
-        <v>2417.13</v>
+        <v>42471.29</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>2293.84</v>
+        <v>38283.74</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>1821.57</v>
-      </c>
-      <c r="L32" s="6" t="n"/>
+        <v>49252.73</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M32" s="5" t="n">
-        <v>1343.95</v>
+        <v>46958.48</v>
       </c>
       <c r="N32" s="5" t="n">
-        <v>1346.02</v>
-      </c>
-      <c r="O32" s="7" t="n">
-        <v>26938.76</v>
+        <v>37271.87</v>
+      </c>
+      <c r="O32" s="6" t="n">
+        <v>423444.27</v>
       </c>
     </row>
     <row r="33">
@@ -1825,45 +2022,47 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>LPS - Production</t>
+          <t>WIMS - Production</t>
         </is>
       </c>
       <c r="C33" s="5" t="n">
-        <v>4259.47</v>
+        <v>2267</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>3716.68</v>
+        <v>2347.5</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>3512.8</v>
+        <v>2194.29</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>3901.6</v>
+        <v>2446.57</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>3192.49</v>
+        <v>2267.4</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>3649.14</v>
+        <v>2267.43</v>
       </c>
       <c r="I33" s="5" t="n">
-        <v>4025.44</v>
+        <v>2555.71</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>3353</v>
+        <v>2078.97</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>4049.53</v>
-      </c>
-      <c r="L33" s="6" t="n"/>
+        <v>2435.78</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M33" s="5" t="n">
-        <v>3701.64</v>
+        <v>2267.43</v>
       </c>
       <c r="N33" s="5" t="n">
-        <v>3228.58</v>
-      </c>
-      <c r="O33" s="7" t="n">
-        <v>40590.38</v>
+        <v>1920.22</v>
+      </c>
+      <c r="O33" s="6" t="n">
+        <v>25048.29</v>
       </c>
     </row>
     <row r="34">
@@ -1874,45 +2073,47 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>NA Frontline - Production</t>
+          <t>Permitted Adjustments</t>
         </is>
       </c>
       <c r="C34" s="5" t="n">
-        <v>16273.82</v>
+        <v>4259.55</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>24548.62</v>
+        <v>3232.15</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>34857.61</v>
+        <v>3874.29</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>36645.12</v>
+        <v>7363.5</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>48700.41</v>
+        <v>7212.28</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>48180.59</v>
+        <v>10333.09</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>42471.29</v>
+        <v>10537.49</v>
       </c>
       <c r="J34" s="5" t="n">
-        <v>38283.74</v>
+        <v>11541.01</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>49252.73</v>
-      </c>
-      <c r="L34" s="6" t="n"/>
+        <v>15754.05</v>
+      </c>
+      <c r="L34" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M34" s="5" t="n">
-        <v>46958.48</v>
+        <v>15019.9</v>
       </c>
       <c r="N34" s="5" t="n">
-        <v>37271.87</v>
-      </c>
-      <c r="O34" s="7" t="n">
-        <v>423444.27</v>
+        <v>12439.23</v>
+      </c>
+      <c r="O34" s="6" t="n">
+        <v>101566.54</v>
       </c>
     </row>
     <row r="35">
@@ -1923,45 +2124,47 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>WIMS - Production</t>
+          <t>Digital Sales</t>
         </is>
       </c>
       <c r="C35" s="5" t="n">
-        <v>2267</v>
+        <v>0</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>2347.5</v>
+        <v>0</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>2194.29</v>
+        <v>3182.23</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>2446.57</v>
+        <v>5513.37</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>2267.4</v>
+        <v>6583.62</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>2267.43</v>
+        <v>5919.16</v>
       </c>
       <c r="I35" s="5" t="n">
-        <v>2555.71</v>
+        <v>5967.17</v>
       </c>
       <c r="J35" s="5" t="n">
-        <v>2078.97</v>
+        <v>8911.450000000001</v>
       </c>
       <c r="K35" s="5" t="n">
-        <v>2435.78</v>
-      </c>
-      <c r="L35" s="6" t="n"/>
+        <v>14637.92</v>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M35" s="5" t="n">
-        <v>2267.43</v>
+        <v>12148.64</v>
       </c>
       <c r="N35" s="5" t="n">
-        <v>1920.22</v>
-      </c>
-      <c r="O35" s="7" t="n">
-        <v>25048.29</v>
+        <v>8313.15</v>
+      </c>
+      <c r="O35" s="6" t="n">
+        <v>71176.71000000001</v>
       </c>
     </row>
     <row r="36">
@@ -1972,45 +2175,47 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Permitted Adjustments</t>
+          <t>Customer Payments</t>
         </is>
       </c>
       <c r="C36" s="5" t="n">
-        <v>4259.55</v>
+        <v>0</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>3232.15</v>
+        <v>0</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>3874.29</v>
+        <v>758.5700000000001</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>7363.5</v>
+        <v>805.42</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>7212.28</v>
+        <v>531.4</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>10333.09</v>
+        <v>531.4299999999999</v>
       </c>
       <c r="I36" s="5" t="n">
-        <v>10537.49</v>
+        <v>611.4</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>11541.01</v>
+        <v>496.74</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>15754.05</v>
-      </c>
-      <c r="L36" s="6" t="n"/>
+        <v>569.73</v>
+      </c>
+      <c r="L36" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M36" s="5" t="n">
-        <v>15019.9</v>
+        <v>32</v>
       </c>
       <c r="N36" s="5" t="n">
-        <v>12439.23</v>
-      </c>
-      <c r="O36" s="7" t="n">
-        <v>101566.54</v>
+        <v>0</v>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>4336.69</v>
       </c>
     </row>
     <row r="37">
@@ -2021,41 +2226,47 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Digital Sales</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
+          <t>WFM Support</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E37" s="5" t="n">
-        <v>3182.23</v>
+        <v>0</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>5513.37</v>
+        <v>256</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>6583.62</v>
+        <v>300</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>5919.16</v>
+        <v>312</v>
       </c>
       <c r="I37" s="5" t="n">
-        <v>5967.17</v>
+        <v>458.3</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>8911.450000000001</v>
+        <v>320</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>14637.92</v>
-      </c>
-      <c r="L37" s="6" t="n"/>
+        <v>394.3</v>
+      </c>
+      <c r="L37" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M37" s="5" t="n">
-        <v>12148.64</v>
+        <v>354.29</v>
       </c>
       <c r="N37" s="5" t="n">
-        <v>8313.15</v>
-      </c>
-      <c r="O37" s="7" t="n">
-        <v>71176.71000000001</v>
+        <v>382.86</v>
+      </c>
+      <c r="O37" s="6" t="n">
+        <v>2777.74</v>
       </c>
     </row>
     <row r="38">
@@ -2066,41 +2277,47 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Customer Payments</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
+          <t>NA RPOps &amp; STOps</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E38" s="5" t="n">
-        <v>758.5700000000001</v>
+        <v>0</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>805.42</v>
+        <v>0</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>531.4</v>
+        <v>0</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>531.4299999999999</v>
+        <v>0</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>611.4</v>
+        <v>0</v>
       </c>
       <c r="J38" s="5" t="n">
-        <v>496.74</v>
+        <v>0</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>569.73</v>
-      </c>
-      <c r="L38" s="6" t="n"/>
+        <v>6876.42</v>
+      </c>
+      <c r="L38" s="5" t="n">
+        <v>6733.52</v>
+      </c>
       <c r="M38" s="5" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="N38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="7" t="n">
-        <v>4336.69</v>
+        <v>6405.72</v>
+      </c>
+      <c r="O38" s="6" t="n">
+        <v>20015.65</v>
       </c>
     </row>
     <row r="39">
@@ -2111,39 +2328,47 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>WFM Support</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
+          <t>RMT - Production</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>1608.72</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="F39" s="5" t="n">
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>312</v>
+        <v>0</v>
       </c>
       <c r="I39" s="5" t="n">
-        <v>458.3</v>
+        <v>0</v>
       </c>
       <c r="J39" s="5" t="n">
-        <v>320</v>
+        <v>0</v>
       </c>
       <c r="K39" s="5" t="n">
-        <v>394.3</v>
-      </c>
-      <c r="L39" s="6" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="L39" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M39" s="5" t="n">
-        <v>354.29</v>
+        <v>0</v>
       </c>
       <c r="N39" s="5" t="n">
-        <v>382.86</v>
-      </c>
-      <c r="O39" s="7" t="n">
-        <v>2777.74</v>
+        <v>0</v>
+      </c>
+      <c r="O39" s="6" t="n">
+        <v>1608.72</v>
       </c>
     </row>
     <row r="40">
@@ -2154,31 +2379,47 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>NA RPOps &amp; STOps</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="6" t="n"/>
+          <t>Finance Team</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>739.9</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="J40" s="5" t="n">
         <v>0</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>6876.42</v>
+        <v>0</v>
       </c>
       <c r="L40" s="5" t="n">
-        <v>6733.52</v>
-      </c>
-      <c r="M40" s="6" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="M40" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="N40" s="5" t="n">
-        <v>6405.72</v>
-      </c>
-      <c r="O40" s="7" t="n">
-        <v>20015.65</v>
+        <v>0</v>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>739.9</v>
       </c>
     </row>
     <row r="41">
@@ -2189,189 +2430,139 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>RMT - Production</t>
+          <t>NA Analytics</t>
         </is>
       </c>
       <c r="C41" s="5" t="n">
-        <v>1608.72</v>
-      </c>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" s="6" t="n"/>
-      <c r="H41" s="6" t="n"/>
-      <c r="I41" s="6" t="n"/>
-      <c r="J41" s="6" t="n"/>
-      <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
-      <c r="M41" s="6" t="n"/>
-      <c r="N41" s="6" t="n"/>
-      <c r="O41" s="7" t="n">
-        <v>1608.72</v>
+        <v>0</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="5" t="n">
+        <v>944</v>
+      </c>
+      <c r="O41" s="6" t="n">
+        <v>944</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>India</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Finance Team</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="5" t="n">
-        <v>739.9</v>
-      </c>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="6" t="n"/>
-      <c r="J42" s="6" t="n"/>
-      <c r="K42" s="6" t="n"/>
-      <c r="L42" s="6" t="n"/>
-      <c r="M42" s="6" t="n"/>
-      <c r="N42" s="6" t="n"/>
-      <c r="O42" s="7" t="n">
-        <v>739.9</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>NA Analytics</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
-      <c r="G43" s="6" t="n"/>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="6" t="n"/>
-      <c r="J43" s="6" t="n"/>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="6" t="n"/>
-      <c r="M43" s="6" t="n"/>
-      <c r="N43" s="5" t="n">
-        <v>944</v>
-      </c>
-      <c r="O43" s="7" t="n">
-        <v>944</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>India</t>
-        </is>
-      </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>India Total</t>
         </is>
       </c>
-      <c r="C44" s="9" t="n">
+      <c r="C42" s="8" t="n">
         <v>32865.97</v>
       </c>
-      <c r="D44" s="9" t="n">
+      <c r="D42" s="8" t="n">
         <v>38249.45</v>
       </c>
-      <c r="E44" s="9" t="n">
+      <c r="E42" s="8" t="n">
         <v>51118.69</v>
       </c>
-      <c r="F44" s="9" t="n">
+      <c r="F42" s="8" t="n">
         <v>59388.98</v>
       </c>
-      <c r="G44" s="9" t="n">
+      <c r="G42" s="8" t="n">
         <v>70930.10000000001</v>
       </c>
-      <c r="H44" s="9" t="n">
+      <c r="H42" s="8" t="n">
         <v>73708.27</v>
       </c>
-      <c r="I44" s="9" t="n">
+      <c r="I42" s="8" t="n">
         <v>69043.92999999999</v>
       </c>
-      <c r="J44" s="9" t="n">
+      <c r="J42" s="8" t="n">
         <v>67278.75</v>
       </c>
-      <c r="K44" s="9" t="n">
+      <c r="K42" s="8" t="n">
         <v>95792.03</v>
       </c>
-      <c r="L44" s="9" t="n">
+      <c r="L42" s="8" t="n">
         <v>6733.52</v>
       </c>
-      <c r="M44" s="9" t="n">
+      <c r="M42" s="8" t="n">
         <v>81826.34</v>
       </c>
-      <c r="N44" s="9" t="n">
+      <c r="N42" s="8" t="n">
         <v>72251.64</v>
       </c>
-      <c r="O44" s="9" t="n">
+      <c r="O42" s="8" t="n">
         <v>719187.66</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>- Values = "Hrs. Billable" total per LOB (col G in 2025 files / col F in 2026 files; located by header).</t>
+        </is>
+      </c>
+    </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>Notes:</t>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>- Blanks shown as 0. All-zero LOB rows (e.g. Egypt GPS) dropped.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>- Values = "Hrs. Billable" total per LOB (col G in 2025 files / col F in 2026 files; located by header).</t>
+          <t>- Duplicate LOB rows within a month (e.g. India WIMS Dec additional billing) are summed.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>- Duplicate LOB rows within a month (e.g. India WIMS "additional billing" catch-up) are summed.</t>
+          <t>- Jamaica: Dec 2025 not provided; Feb 2026 file is B2C-only. Canada: only Sep 2025 - Feb 2026 provided.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>- Jamaica: Dec 2025 not provided; Feb 2026 file is B2C-only (other LOBs blank).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>- Canada: only Sep 2025 - Feb 2026 provided.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>- India: Apr 2026 file is GPS/RPOps-only - only "NA RPOps &amp; STOps" populated; service LOBs blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>- India Oct 2025: used the v2 (revised) file.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>- Blank cell = LOB not present / no data in that month file.</t>
+          <t>- India: Apr 2026 file is GPS/RPOps-only (only NA RPOps &amp; STOps populated). Oct 2025 used v2 file.</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2405,7 +2596,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Jamaica - Production Hours Billable by LOB and Month</t>
         </is>
@@ -2502,7 +2693,9 @@
       <c r="G4" s="5" t="n">
         <v>59150.74</v>
       </c>
-      <c r="H4" s="6" t="n"/>
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" s="5" t="n">
         <v>43959.67</v>
       </c>
@@ -2515,7 +2708,7 @@
       <c r="L4" s="5" t="n">
         <v>33943.17</v>
       </c>
-      <c r="M4" s="7" t="n">
+      <c r="M4" s="6" t="n">
         <v>442918.69</v>
       </c>
     </row>
@@ -2543,7 +2736,9 @@
       <c r="G5" s="5" t="n">
         <v>7390.85</v>
       </c>
-      <c r="H5" s="6" t="n"/>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" s="5" t="n">
         <v>5300.01</v>
       </c>
@@ -2556,7 +2751,7 @@
       <c r="L5" s="5" t="n">
         <v>145.97</v>
       </c>
-      <c r="M5" s="7" t="n">
+      <c r="M5" s="6" t="n">
         <v>100444.69</v>
       </c>
     </row>
@@ -2584,7 +2779,9 @@
       <c r="G6" s="5" t="n">
         <v>7964.95</v>
       </c>
-      <c r="H6" s="6" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" s="5" t="n">
         <v>9913.139999999999</v>
       </c>
@@ -2597,7 +2794,7 @@
       <c r="L6" s="5" t="n">
         <v>7413.2</v>
       </c>
-      <c r="M6" s="7" t="n">
+      <c r="M6" s="6" t="n">
         <v>66573.32000000001</v>
       </c>
     </row>
@@ -2625,7 +2822,9 @@
       <c r="G7" s="5" t="n">
         <v>4194.25</v>
       </c>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" s="5" t="n">
         <v>4833.93</v>
       </c>
@@ -2638,7 +2837,7 @@
       <c r="L7" s="5" t="n">
         <v>10320.62</v>
       </c>
-      <c r="M7" s="7" t="n">
+      <c r="M7" s="6" t="n">
         <v>58307.27</v>
       </c>
     </row>
@@ -2648,17 +2847,27 @@
           <t>NA LPAX Voice - Production</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="F8" s="5" t="n">
         <v>2881.93</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>3761.51</v>
       </c>
-      <c r="H8" s="6" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="5" t="n">
         <v>3714.27</v>
       </c>
@@ -2671,7 +2880,7 @@
       <c r="L8" s="5" t="n">
         <v>4713.46</v>
       </c>
-      <c r="M8" s="7" t="n">
+      <c r="M8" s="6" t="n">
         <v>20763.51</v>
       </c>
     </row>
@@ -2681,12 +2890,24 @@
           <t>B2C - Production</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="5" t="n">
         <v>1622.5</v>
       </c>
@@ -2699,74 +2920,53 @@
       <c r="K9" s="5" t="n">
         <v>1038.75</v>
       </c>
-      <c r="L9" s="6" t="n"/>
-      <c r="M9" s="7" t="n">
+      <c r="L9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6" t="n">
         <v>3164.33</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>WIMS - Production</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="n"/>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
-      <c r="M10" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>60570.3</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C10" s="8" t="n">
         <v>60849.45</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D10" s="8" t="n">
         <v>59022.47</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E10" s="8" t="n">
         <v>68545.72</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F10" s="8" t="n">
         <v>96107.10000000001</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G10" s="8" t="n">
         <v>82462.3</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H10" s="8" t="n">
         <v>1622.5</v>
       </c>
-      <c r="I11" s="9" t="n">
+      <c r="I10" s="8" t="n">
         <v>68063.92</v>
       </c>
-      <c r="J11" s="9" t="n">
+      <c r="J10" s="8" t="n">
         <v>72325.08</v>
       </c>
-      <c r="K11" s="9" t="n">
+      <c r="K10" s="8" t="n">
         <v>66066.56</v>
       </c>
-      <c r="L11" s="9" t="n">
+      <c r="L10" s="8" t="n">
         <v>56536.41</v>
       </c>
-      <c r="M11" s="9" t="n">
+      <c r="M10" s="8" t="n">
         <v>692171.8100000001</v>
       </c>
     </row>
@@ -2781,7 +2981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2801,7 +3001,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Egypt - Production Hours Billable by LOB and Month</t>
         </is>
@@ -2921,7 +3121,7 @@
       <c r="M4" s="5" t="n">
         <v>10879.47</v>
       </c>
-      <c r="N4" s="7" t="n">
+      <c r="N4" s="6" t="n">
         <v>176564.73</v>
       </c>
     </row>
@@ -2967,7 +3167,7 @@
       <c r="M5" s="5" t="n">
         <v>4276.37</v>
       </c>
-      <c r="N5" s="7" t="n">
+      <c r="N5" s="6" t="n">
         <v>68679.72</v>
       </c>
     </row>
@@ -2977,8 +3177,12 @@
           <t>ESL NA Digital Sales - Production</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D6" s="5" t="n">
         <v>1540.21</v>
       </c>
@@ -2991,7 +3195,9 @@
       <c r="G6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="6" t="n"/>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" s="5" t="n">
         <v>1893.36</v>
       </c>
@@ -3007,7 +3213,7 @@
       <c r="M6" s="5" t="n">
         <v>1747.12</v>
       </c>
-      <c r="N6" s="7" t="n">
+      <c r="N6" s="6" t="n">
         <v>12522.88</v>
       </c>
     </row>
@@ -3017,8 +3223,12 @@
           <t>CA FR Voice - Production</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D7" s="5" t="n">
         <v>2048.13</v>
       </c>
@@ -3049,7 +3259,7 @@
       <c r="M7" s="5" t="n">
         <v>1811.12</v>
       </c>
-      <c r="N7" s="7" t="n">
+      <c r="N7" s="6" t="n">
         <v>25222.55</v>
       </c>
     </row>
@@ -3059,8 +3269,12 @@
           <t>ESL UK Digital Sales - Production</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="6" t="n"/>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D8" s="5" t="n">
         <v>1789.5</v>
       </c>
@@ -3091,7 +3305,7 @@
       <c r="M8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="7" t="n">
+      <c r="N8" s="6" t="n">
         <v>1789.5</v>
       </c>
     </row>
@@ -3101,8 +3315,12 @@
           <t>ESL NA Voice Sales - Production</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D9" s="5" t="n">
         <v>2528.78</v>
       </c>
@@ -3133,7 +3351,7 @@
       <c r="M9" s="5" t="n">
         <v>9621.950000000001</v>
       </c>
-      <c r="N9" s="7" t="n">
+      <c r="N9" s="6" t="n">
         <v>106124.15</v>
       </c>
     </row>
@@ -3143,8 +3361,12 @@
           <t>ESL UK Voice Service - Production</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D10" s="5" t="n">
         <v>2971.44</v>
       </c>
@@ -3175,7 +3397,7 @@
       <c r="M10" s="5" t="n">
         <v>4931.92</v>
       </c>
-      <c r="N10" s="7" t="n">
+      <c r="N10" s="6" t="n">
         <v>48141.35</v>
       </c>
     </row>
@@ -3185,8 +3407,12 @@
           <t>ESL UK Voice Sales - Production</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D11" s="5" t="n">
         <v>2171.57</v>
       </c>
@@ -3217,7 +3443,7 @@
       <c r="M11" s="5" t="n">
         <v>1276.85</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="N11" s="6" t="n">
         <v>22846.7</v>
       </c>
     </row>
@@ -3227,8 +3453,12 @@
           <t>ESL SP Voice Service - Production</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D12" s="5" t="n">
         <v>876.1799999999999</v>
       </c>
@@ -3259,7 +3489,7 @@
       <c r="M12" s="5" t="n">
         <v>1651.05</v>
       </c>
-      <c r="N12" s="7" t="n">
+      <c r="N12" s="6" t="n">
         <v>25739.05</v>
       </c>
     </row>
@@ -3269,10 +3499,18 @@
           <t>ESL NA LPAX Voice Service - Production</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
+      <c r="B13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="F13" s="5" t="n">
         <v>0</v>
       </c>
@@ -3297,7 +3535,7 @@
       <c r="M13" s="5" t="n">
         <v>3198.53</v>
       </c>
-      <c r="N13" s="7" t="n">
+      <c r="N13" s="6" t="n">
         <v>29481.52</v>
       </c>
     </row>
@@ -3307,12 +3545,24 @@
           <t>ESL NA Voice Service - Production</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="H14" s="5" t="n">
         <v>997.02</v>
       </c>
@@ -3331,7 +3581,7 @@
       <c r="M14" s="5" t="n">
         <v>26567.43</v>
       </c>
-      <c r="N14" s="7" t="n">
+      <c r="N14" s="6" t="n">
         <v>116422.51</v>
       </c>
     </row>
@@ -3341,10 +3591,18 @@
           <t>ESL UK Voice Service DHD - Production</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="F15" s="5" t="n">
         <v>0</v>
       </c>
@@ -3369,7 +3627,7 @@
       <c r="M15" s="5" t="n">
         <v>2334.82</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="6" t="n">
         <v>16826.76</v>
       </c>
     </row>
@@ -3379,13 +3637,27 @@
           <t>French Sales - Production</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
+      <c r="B16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I16" s="5" t="n">
         <v>839.76</v>
       </c>
@@ -3401,7 +3673,7 @@
       <c r="M16" s="5" t="n">
         <v>1506.23</v>
       </c>
-      <c r="N16" s="7" t="n">
+      <c r="N16" s="6" t="n">
         <v>7792.96</v>
       </c>
     </row>
@@ -3411,13 +3683,27 @@
           <t>Spanish Sales - Production</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
+      <c r="B17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I17" s="5" t="n">
         <v>828.1</v>
       </c>
@@ -3433,23 +3719,37 @@
       <c r="M17" s="5" t="n">
         <v>1688.9</v>
       </c>
-      <c r="N17" s="7" t="n">
+      <c r="N17" s="6" t="n">
         <v>8152.52</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>GPS - Production</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
+          <t>ESL Digital Sales - Production</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>2357.05</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>2127</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I18" s="5" t="n">
         <v>0</v>
       </c>
@@ -3465,79 +3765,53 @@
       <c r="M18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N18" s="7" t="n">
-        <v>0</v>
+      <c r="N18" s="6" t="n">
+        <v>4484.05</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>ESL Digital Sales - Production</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>2357.05</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>2127</v>
-      </c>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="6" t="n"/>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="6" t="n"/>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="7" t="n">
-        <v>4484.05</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B19" s="8" t="n">
         <v>9310.82</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C19" s="8" t="n">
         <v>8176</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D19" s="8" t="n">
         <v>26445.9</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E19" s="8" t="n">
         <v>43506.64</v>
       </c>
-      <c r="F20" s="9" t="n">
+      <c r="F19" s="8" t="n">
         <v>48276.24</v>
       </c>
-      <c r="G20" s="9" t="n">
+      <c r="G19" s="8" t="n">
         <v>58518.33</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="H19" s="8" t="n">
         <v>61268.47</v>
       </c>
-      <c r="I20" s="9" t="n">
+      <c r="I19" s="8" t="n">
         <v>74747</v>
       </c>
-      <c r="J20" s="9" t="n">
+      <c r="J19" s="8" t="n">
         <v>92947.50999999999</v>
       </c>
-      <c r="K20" s="9" t="n">
+      <c r="K19" s="8" t="n">
         <v>88632.53999999999</v>
       </c>
-      <c r="L20" s="9" t="n">
+      <c r="L19" s="8" t="n">
         <v>87469.74000000001</v>
       </c>
-      <c r="M20" s="9" t="n">
+      <c r="M19" s="8" t="n">
         <v>71491.75</v>
       </c>
-      <c r="N20" s="9" t="n">
+      <c r="N19" s="8" t="n">
         <v>670790.9399999999</v>
       </c>
     </row>
@@ -3566,7 +3840,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Canada - Production Hours Billable by LOB and Month</t>
         </is>
@@ -3638,35 +3912,35 @@
       <c r="G4" s="5" t="n">
         <v>396.94</v>
       </c>
-      <c r="H4" s="7" t="n">
+      <c r="H4" s="6" t="n">
         <v>10519.58</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>2073.63</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>2230.7</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>1712</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="8" t="n">
         <v>2113.83</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F5" s="8" t="n">
         <v>1992.48</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="8" t="n">
         <v>396.94</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="8" t="n">
         <v>10519.58</v>
       </c>
     </row>
@@ -3701,7 +3975,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>India - Production Hours Billable by LOB and Month</t>
         </is>
@@ -3812,14 +4086,16 @@
       <c r="J4" s="5" t="n">
         <v>1821.57</v>
       </c>
-      <c r="K4" s="6" t="n"/>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L4" s="5" t="n">
         <v>1343.95</v>
       </c>
       <c r="M4" s="5" t="n">
         <v>1346.02</v>
       </c>
-      <c r="N4" s="7" t="n">
+      <c r="N4" s="6" t="n">
         <v>26938.76</v>
       </c>
     </row>
@@ -3856,14 +4132,16 @@
       <c r="J5" s="5" t="n">
         <v>4049.53</v>
       </c>
-      <c r="K5" s="6" t="n"/>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L5" s="5" t="n">
         <v>3701.64</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>3228.58</v>
       </c>
-      <c r="N5" s="7" t="n">
+      <c r="N5" s="6" t="n">
         <v>40590.38</v>
       </c>
     </row>
@@ -3900,14 +4178,16 @@
       <c r="J6" s="5" t="n">
         <v>49252.73</v>
       </c>
-      <c r="K6" s="6" t="n"/>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L6" s="5" t="n">
         <v>46958.48</v>
       </c>
       <c r="M6" s="5" t="n">
         <v>37271.87</v>
       </c>
-      <c r="N6" s="7" t="n">
+      <c r="N6" s="6" t="n">
         <v>423444.27</v>
       </c>
     </row>
@@ -3944,14 +4224,16 @@
       <c r="J7" s="5" t="n">
         <v>2435.78</v>
       </c>
-      <c r="K7" s="6" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L7" s="5" t="n">
         <v>2267.43</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>1920.22</v>
       </c>
-      <c r="N7" s="7" t="n">
+      <c r="N7" s="6" t="n">
         <v>25048.29</v>
       </c>
     </row>
@@ -3988,14 +4270,16 @@
       <c r="J8" s="5" t="n">
         <v>15754.05</v>
       </c>
-      <c r="K8" s="6" t="n"/>
+      <c r="K8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L8" s="5" t="n">
         <v>15019.9</v>
       </c>
       <c r="M8" s="5" t="n">
         <v>12439.23</v>
       </c>
-      <c r="N8" s="7" t="n">
+      <c r="N8" s="6" t="n">
         <v>101566.54</v>
       </c>
     </row>
@@ -4005,8 +4289,12 @@
           <t>Digital Sales</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D9" s="5" t="n">
         <v>3182.23</v>
       </c>
@@ -4028,14 +4316,16 @@
       <c r="J9" s="5" t="n">
         <v>14637.92</v>
       </c>
-      <c r="K9" s="6" t="n"/>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L9" s="5" t="n">
         <v>12148.64</v>
       </c>
       <c r="M9" s="5" t="n">
         <v>8313.15</v>
       </c>
-      <c r="N9" s="7" t="n">
+      <c r="N9" s="6" t="n">
         <v>71176.71000000001</v>
       </c>
     </row>
@@ -4045,8 +4335,12 @@
           <t>Customer Payments</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="D10" s="5" t="n">
         <v>758.5700000000001</v>
       </c>
@@ -4068,14 +4362,16 @@
       <c r="J10" s="5" t="n">
         <v>569.73</v>
       </c>
-      <c r="K10" s="6" t="n"/>
+      <c r="K10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="5" t="n">
         <v>32</v>
       </c>
       <c r="M10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="7" t="n">
+      <c r="N10" s="6" t="n">
         <v>4336.69</v>
       </c>
     </row>
@@ -4085,9 +4381,15 @@
           <t>WFM Support</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
+      <c r="B11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E11" s="5" t="n">
         <v>256</v>
       </c>
@@ -4106,14 +4408,16 @@
       <c r="J11" s="5" t="n">
         <v>394.3</v>
       </c>
-      <c r="K11" s="6" t="n"/>
+      <c r="K11" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L11" s="5" t="n">
         <v>354.29</v>
       </c>
       <c r="M11" s="5" t="n">
         <v>382.86</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="N11" s="6" t="n">
         <v>2777.74</v>
       </c>
     </row>
@@ -4123,13 +4427,27 @@
           <t>NA RPOps &amp; STOps</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
+      <c r="B12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="I12" s="5" t="n">
         <v>0</v>
       </c>
@@ -4139,11 +4457,13 @@
       <c r="K12" s="5" t="n">
         <v>6733.52</v>
       </c>
-      <c r="L12" s="6" t="n"/>
+      <c r="L12" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M12" s="5" t="n">
         <v>6405.72</v>
       </c>
-      <c r="N12" s="7" t="n">
+      <c r="N12" s="6" t="n">
         <v>20015.65</v>
       </c>
     </row>
@@ -4156,18 +4476,40 @@
       <c r="B13" s="5" t="n">
         <v>1608.72</v>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="7" t="n">
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="6" t="n">
         <v>1608.72</v>
       </c>
     </row>
@@ -4177,21 +4519,43 @@
           <t>Finance Team</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n"/>
+      <c r="B14" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="C14" s="5" t="n">
         <v>739.9</v>
       </c>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="n"/>
-      <c r="K14" s="6" t="n"/>
-      <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6" t="n"/>
-      <c r="N14" s="7" t="n">
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="6" t="n">
         <v>739.9</v>
       </c>
     </row>
@@ -4201,67 +4565,89 @@
           <t>NA Analytics</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
+      <c r="B15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="M15" s="5" t="n">
         <v>944</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="6" t="n">
         <v>944</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="8" t="n">
         <v>32865.97</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="8" t="n">
         <v>38249.45</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="8" t="n">
         <v>51118.69</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="8" t="n">
         <v>59388.98</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F16" s="8" t="n">
         <v>70930.10000000001</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G16" s="8" t="n">
         <v>73708.27</v>
       </c>
-      <c r="H16" s="9" t="n">
+      <c r="H16" s="8" t="n">
         <v>69043.92999999999</v>
       </c>
-      <c r="I16" s="9" t="n">
+      <c r="I16" s="8" t="n">
         <v>67278.75</v>
       </c>
-      <c r="J16" s="9" t="n">
+      <c r="J16" s="8" t="n">
         <v>95792.03</v>
       </c>
-      <c r="K16" s="9" t="n">
+      <c r="K16" s="8" t="n">
         <v>6733.52</v>
       </c>
-      <c r="L16" s="9" t="n">
+      <c r="L16" s="8" t="n">
         <v>81826.34</v>
       </c>
-      <c r="M16" s="9" t="n">
+      <c r="M16" s="8" t="n">
         <v>72251.64</v>
       </c>
-      <c r="N16" s="9" t="n">
+      <c r="N16" s="8" t="n">
         <v>719187.66</v>
       </c>
     </row>

</xml_diff>